<commit_message>
added 'game end' and OE bonus card translation in FR
</commit_message>
<xml_diff>
--- a/i18n/fr.xlsx
+++ b/i18n/fr.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="23901"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10509"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matej\Programming\wingsearch\i18n\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Touniouk/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81C963F6-9633-437E-A625-07E96FDB0C79}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BA8BB50-FAA1-7544-A903-CEA0DD101E84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="19720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Birds" sheetId="1" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2222" uniqueCount="1524">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2245" uniqueCount="1543">
   <si>
     <t>id</t>
   </si>
@@ -3806,6 +3806,9 @@
     <t>Défaussez 1 [egg] d’un de vos autres oiseaux pour gagner 2 [wild] de la réserve.</t>
   </si>
   <si>
+    <t>Choisissez 1 autre joueur. Pour chaque cube Action sur sa ligne [grasslandd], glissez 1 [card] de votre main sous cet oiseau, puis piochez autant de [card].</t>
+  </si>
+  <si>
     <t>Vous pouvez glisser des cartes à concurrence du nombre de cubes Action.</t>
   </si>
   <si>
@@ -3816,6 +3819,9 @@
   </si>
   <si>
     <t>Les nids [star] comptent comme des [bowl] ou [ground] pour cet oiseau.</t>
+  </si>
+  <si>
+    <t>Piochez 1 [cardd] face visible qui puisse être jouée dans [wetland].</t>
   </si>
   <si>
     <t>Choisissez 1 à 3 oiseaux dans votre [wetland]. Glissez 1 [card] de votre main sous chacun d’eux. Si vous le faites, piochez 1 [card].</t>
@@ -4474,6 +4480,9 @@
     <t>Faucon Brun</t>
   </si>
   <si>
+    <t>Regardez une [card] de la pioche. Si le coût en nourriture inclut [invertebrate] ou [mouse], glissez-la sous cet oiseau, sinon défaussez-la.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Aigle d'Australie </t>
   </si>
   <si>
@@ -4490,6 +4499,9 @@
   </si>
   <si>
     <t>Élanion d'Australie</t>
+  </si>
+  <si>
+    <t>Relancez les dés de la mangeoire et gagnez 1 [rodednt], si disponible. Vous pouvez le donner à un autre joueur. Si vous le faites, pondez jusqu'à 3 [egg] sur cet oiseau.</t>
   </si>
   <si>
     <t xml:space="preserve">Pitohui Gris </t>
@@ -4683,16 +4695,66 @@
     <t>Vautour des palombes</t>
   </si>
   <si>
-    <t>Piochez 1 [card] face visible qui puisse être jouée dans [wetland].</t>
-  </si>
-  <si>
-    <t>Regardez une [card] de la pioche. Si le coût en nourriture inclut [invertebrate] ou [rodent], glissez-la sous cet oiseau, sinon défaussez-la.</t>
-  </si>
-  <si>
-    <t>Relancez les dés de la mangeoire et gagnez 1 [rodent], si disponible. Vous pouvez le donner à un autre joueur. Si vous le faites, pondez jusqu'à 3 [egg] sur cet oiseau.</t>
-  </si>
-  <si>
-    <t>Choisissez 1 autre joueur. Pour chaque cube Action sur sa ligne [grassland], glissez 1 [card] de votre main sous cet oiseau, puis piochez autant de [card].</t>
+    <t>FIN DE PARTIE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ingénieur Mécanique </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cette carte vous fait marquer des points pour chaque série de 4 nids de types différents parmi vos oiseaux. L’ordre et l’emplacement des nids sont sans importance, chaque série doit juste contenir un nid de chacun des quatre types. </t>
+  </si>
+  <si>
+    <t>Les nids étoile sont des jokers, ils comptent comme des nids du type de votre choix. Chaque carte ne compte que pour une série.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Séries de nids de 4 types différents </t>
+  </si>
+  <si>
+    <t>1 série: 3[point]; 2+ séries: 8[point]</t>
+  </si>
+  <si>
+    <t>Expert en choix d'emplacement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Colonnes avec deux ou trois nids du même type </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Le type de nid peut être différent d’une colonne à l’autre. Les nids étoile sont des jokers, mais chacun ne compte qu’une fois. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyste de données marécageuses </t>
+  </si>
+  <si>
+    <t>Analyste de données prairiales</t>
+  </si>
+  <si>
+    <t>Analyste de données forestières</t>
+  </si>
+  <si>
+    <t>Ces cartes Bonus vous font gagner des points pour les suites d’oiseaux dans l’habitat correspondant avec une envergure
+croissante ou décroissante. La suite ne comprend pas obligatoirement tous les oiseaux de l’habitat. Elle n’est pas tenue de commencer ou de finir avec le premier et le dernier oiseau
+de cet habitat. Une suite peut contenir deux oiseaux ou plus avec la même envergure.
+Comme indiqué précédemment, les oiseaux inaptes au vol sont des jokers : vous pouvez choisir l’envergure des oiseaux inaptes au vol lors du calcul des points de ces cartes bonus.
+Par exemple, si l’envergure des 3 premiers oiseaux de votre marais est croissante, mais que le 4ème oiseau dans cet habitat a une envergure inférieure au 3ème, vous avez une suite de 3 cartes et vous gagnez 3 points grâce à la carte Bonus Analyste de données marécageuses.</t>
+  </si>
+  <si>
+    <t>Suite d'oiseaux dans [grassland] avec une envergure croissante ou décroissante</t>
+  </si>
+  <si>
+    <t>Suite d'oiseaux dans [wetland] avec une envergure croissante ou décroissante</t>
+  </si>
+  <si>
+    <t>Suite d'oiseaux dans [forest] avec une envergure croissante ou décroissante</t>
+  </si>
+  <si>
+    <t>Cette carte Bonus vous fait gagner des points pour chaque colonne contenant plus d’un nid du même type. Une colonne vous fait gagner 0, 1 ou 3 points selon le nombre de nids identiques dans cette colonne (0 points si tous les nids sont différents, 1 points si vous avez 2 nids identiques, 3 points si les 3 nids sont identiques). Le type de nid peut être différent d’une colonne à l’autre.
+Les nids étoile sont des jokers. Chaque nid étoile ne compte qu’une fois et ne peut pas être utilisé pour faire 2 paires dans la même colonne.</t>
+  </si>
+  <si>
+    <t>Suite de 3 oiseaux: 3[point]; Suite de 4 oiseaux: 5[point]; Suite de 5 oiseaux: 8[point];</t>
+  </si>
+  <si>
+    <t>2 nids identiques dans une colonne: 1[point]; 3 nids identiques dans une colonne: 3[point];</t>
   </si>
 </sst>
 </file>
@@ -4778,7 +4840,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -4822,9 +4884,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normálna" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="25">
     <dxf>
@@ -5278,18 +5343,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J357"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="4.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="26.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="4.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="26.1640625" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="43.6640625" style="4" customWidth="1"/>
-    <col min="6" max="6" width="54.109375" style="4" customWidth="1"/>
-    <col min="7" max="10" width="9.109375" style="1" customWidth="1"/>
-    <col min="11" max="16384" width="9.109375" style="1"/>
+    <col min="6" max="6" width="54.1640625" style="4" customWidth="1"/>
+    <col min="7" max="10" width="9.1640625" style="1" customWidth="1"/>
+    <col min="11" max="16384" width="9.1640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="13.95" customHeight="1">
+    <row r="1" spans="1:10" ht="14" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -5799,7 +5864,7 @@
         <v>590</v>
       </c>
       <c r="E20" s="12" t="s">
-        <v>1303</v>
+        <v>1305</v>
       </c>
       <c r="F20" s="12" t="s">
         <v>8</v>
@@ -5977,10 +6042,10 @@
         <v>597</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>1280</v>
+        <v>1282</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>1279</v>
+        <v>1281</v>
       </c>
       <c r="G27" s="14"/>
       <c r="H27" s="14" t="s">
@@ -6029,7 +6094,7 @@
         <v>599</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>1243</v>
+        <v>1245</v>
       </c>
       <c r="F29" s="10" t="s">
         <v>8</v>
@@ -6111,10 +6176,10 @@
         <v>602</v>
       </c>
       <c r="E32" s="12" t="s">
-        <v>1299</v>
+        <v>1301</v>
       </c>
       <c r="F32" s="12" t="s">
-        <v>1300</v>
+        <v>1302</v>
       </c>
       <c r="G32" s="14"/>
       <c r="H32" s="14"/>
@@ -6137,10 +6202,10 @@
         <v>603</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>1296</v>
+        <v>1298</v>
       </c>
       <c r="F33" s="5" t="s">
-        <v>1297</v>
+        <v>1299</v>
       </c>
       <c r="G33" s="14"/>
       <c r="H33" s="14"/>
@@ -6191,10 +6256,10 @@
         <v>605</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>1299</v>
+        <v>1301</v>
       </c>
       <c r="F35" s="5" t="s">
-        <v>1300</v>
+        <v>1302</v>
       </c>
       <c r="G35" s="14"/>
       <c r="H35" s="14" t="s">
@@ -6271,7 +6336,7 @@
         <v>608</v>
       </c>
       <c r="E38" s="10" t="s">
-        <v>1292</v>
+        <v>1294</v>
       </c>
       <c r="F38" s="10" t="s">
         <v>1224</v>
@@ -6295,7 +6360,7 @@
         <v>609</v>
       </c>
       <c r="E39" s="10" t="s">
-        <v>1240</v>
+        <v>1242</v>
       </c>
       <c r="F39" s="10" t="s">
         <v>1214</v>
@@ -6427,7 +6492,7 @@
         <v>614</v>
       </c>
       <c r="E44" s="5" t="s">
-        <v>1252</v>
+        <v>1254</v>
       </c>
       <c r="F44" s="5" t="s">
         <v>8</v>
@@ -6481,7 +6546,7 @@
         <v>616</v>
       </c>
       <c r="E46" s="10" t="s">
-        <v>1253</v>
+        <v>1255</v>
       </c>
       <c r="F46" s="10" t="s">
         <v>8</v>
@@ -6659,7 +6724,7 @@
         <v>623</v>
       </c>
       <c r="E53" s="12" t="s">
-        <v>1294</v>
+        <v>1296</v>
       </c>
       <c r="F53" s="12" t="s">
         <v>8</v>
@@ -6917,7 +6982,7 @@
         <v>633</v>
       </c>
       <c r="E63" s="12" t="s">
-        <v>1240</v>
+        <v>1242</v>
       </c>
       <c r="F63" s="12" t="s">
         <v>1214</v>
@@ -6943,7 +7008,7 @@
         <v>634</v>
       </c>
       <c r="E64" s="12" t="s">
-        <v>1235</v>
+        <v>1236</v>
       </c>
       <c r="F64" s="12" t="s">
         <v>8</v>
@@ -7021,7 +7086,7 @@
         <v>637</v>
       </c>
       <c r="E67" s="12" t="s">
-        <v>1271</v>
+        <v>1273</v>
       </c>
       <c r="F67" s="12" t="s">
         <v>8</v>
@@ -7255,10 +7320,10 @@
         <v>646</v>
       </c>
       <c r="E76" s="5" t="s">
-        <v>1286</v>
+        <v>1288</v>
       </c>
       <c r="F76" s="5" t="s">
-        <v>1287</v>
+        <v>1289</v>
       </c>
       <c r="G76" s="14"/>
       <c r="H76" s="14"/>
@@ -7281,10 +7346,10 @@
         <v>647</v>
       </c>
       <c r="E77" s="10" t="s">
-        <v>1284</v>
+        <v>1286</v>
       </c>
       <c r="F77" s="10" t="s">
-        <v>1269</v>
+        <v>1271</v>
       </c>
       <c r="G77" s="14"/>
       <c r="H77" s="14"/>
@@ -7331,10 +7396,10 @@
         <v>649</v>
       </c>
       <c r="E79" s="12" t="s">
-        <v>1301</v>
+        <v>1303</v>
       </c>
       <c r="F79" s="12" t="s">
-        <v>1302</v>
+        <v>1304</v>
       </c>
       <c r="G79" s="14"/>
       <c r="H79" s="14"/>
@@ -7355,10 +7420,10 @@
         <v>650</v>
       </c>
       <c r="E80" s="11" t="s">
-        <v>1301</v>
+        <v>1303</v>
       </c>
       <c r="F80" s="11" t="s">
-        <v>1302</v>
+        <v>1304</v>
       </c>
       <c r="G80" s="14"/>
       <c r="H80" s="14"/>
@@ -7379,10 +7444,10 @@
         <v>651</v>
       </c>
       <c r="E81" s="5" t="s">
-        <v>1236</v>
+        <v>1237</v>
       </c>
       <c r="F81" s="5" t="s">
-        <v>1237</v>
+        <v>1238</v>
       </c>
       <c r="G81" s="14"/>
       <c r="H81" s="14"/>
@@ -7405,10 +7470,10 @@
         <v>652</v>
       </c>
       <c r="E82" s="5" t="s">
-        <v>1250</v>
+        <v>1252</v>
       </c>
       <c r="F82" s="5" t="s">
-        <v>1251</v>
+        <v>1253</v>
       </c>
       <c r="G82" s="14" t="s">
         <v>1133</v>
@@ -7557,10 +7622,10 @@
         <v>658</v>
       </c>
       <c r="E88" s="5" t="s">
-        <v>1249</v>
+        <v>1251</v>
       </c>
       <c r="F88" s="5" t="s">
-        <v>1246</v>
+        <v>1248</v>
       </c>
       <c r="G88" s="14"/>
       <c r="H88" s="14"/>
@@ -7607,7 +7672,7 @@
         <v>660</v>
       </c>
       <c r="E90" s="10" t="s">
-        <v>1253</v>
+        <v>1255</v>
       </c>
       <c r="F90" s="10" t="s">
         <v>8</v>
@@ -7729,7 +7794,7 @@
         <v>665</v>
       </c>
       <c r="E95" s="12" t="s">
-        <v>1241</v>
+        <v>1243</v>
       </c>
       <c r="F95" s="12" t="s">
         <v>1178</v>
@@ -7755,7 +7820,7 @@
         <v>666</v>
       </c>
       <c r="E96" s="12" t="s">
-        <v>1306</v>
+        <v>1308</v>
       </c>
       <c r="F96" s="12" t="s">
         <v>1185</v>
@@ -7781,7 +7846,7 @@
         <v>667</v>
       </c>
       <c r="E97" s="7" t="s">
-        <v>1273</v>
+        <v>1275</v>
       </c>
       <c r="F97" s="7" t="s">
         <v>8</v>
@@ -7959,10 +8024,10 @@
         <v>674</v>
       </c>
       <c r="E104" s="9" t="s">
+        <v>1283</v>
+      </c>
+      <c r="F104" s="9" t="s">
         <v>1281</v>
-      </c>
-      <c r="F104" s="9" t="s">
-        <v>1279</v>
       </c>
       <c r="G104" s="14"/>
       <c r="H104" s="14"/>
@@ -7983,7 +8048,7 @@
         <v>675</v>
       </c>
       <c r="E105" s="5" t="s">
-        <v>1289</v>
+        <v>1291</v>
       </c>
       <c r="F105" s="5" t="s">
         <v>8</v>
@@ -8031,7 +8096,7 @@
         <v>677</v>
       </c>
       <c r="E107" s="12" t="s">
-        <v>1242</v>
+        <v>1244</v>
       </c>
       <c r="F107" s="12" t="s">
         <v>8</v>
@@ -8083,10 +8148,10 @@
         <v>679</v>
       </c>
       <c r="E109" s="10" t="s">
-        <v>1276</v>
+        <v>1278</v>
       </c>
       <c r="F109" s="10" t="s">
-        <v>1277</v>
+        <v>1279</v>
       </c>
       <c r="G109" s="14"/>
       <c r="H109" s="14" t="s">
@@ -8112,7 +8177,7 @@
         <v>1198</v>
       </c>
       <c r="F110" s="5" t="s">
-        <v>1293</v>
+        <v>1295</v>
       </c>
       <c r="G110" s="14"/>
       <c r="H110" s="14"/>
@@ -8183,7 +8248,7 @@
         <v>683</v>
       </c>
       <c r="E113" s="5" t="s">
-        <v>1298</v>
+        <v>1300</v>
       </c>
       <c r="F113" s="5" t="s">
         <v>1221</v>
@@ -8231,10 +8296,10 @@
         <v>685</v>
       </c>
       <c r="E115" s="5" t="s">
-        <v>1286</v>
+        <v>1288</v>
       </c>
       <c r="F115" s="5" t="s">
-        <v>1287</v>
+        <v>1289</v>
       </c>
       <c r="G115" s="14"/>
       <c r="H115" s="14"/>
@@ -8281,10 +8346,10 @@
         <v>687</v>
       </c>
       <c r="E117" s="7" t="s">
-        <v>1278</v>
+        <v>1280</v>
       </c>
       <c r="F117" s="7" t="s">
-        <v>1277</v>
+        <v>1279</v>
       </c>
       <c r="G117" s="14"/>
       <c r="H117" s="14"/>
@@ -8305,7 +8370,7 @@
         <v>688</v>
       </c>
       <c r="E118" s="5" t="s">
-        <v>1263</v>
+        <v>1265</v>
       </c>
       <c r="F118" s="5" t="s">
         <v>1197</v>
@@ -8379,10 +8444,10 @@
         <v>691</v>
       </c>
       <c r="E121" s="12" t="s">
-        <v>1304</v>
+        <v>1306</v>
       </c>
       <c r="F121" s="12" t="s">
-        <v>1305</v>
+        <v>1307</v>
       </c>
       <c r="G121" s="14" t="s">
         <v>1133</v>
@@ -8407,10 +8472,10 @@
         <v>692</v>
       </c>
       <c r="E122" s="7" t="s">
-        <v>1285</v>
+        <v>1287</v>
       </c>
       <c r="F122" s="7" t="s">
-        <v>1269</v>
+        <v>1271</v>
       </c>
       <c r="G122" s="14"/>
       <c r="H122" s="14" t="s">
@@ -8433,7 +8498,7 @@
         <v>693</v>
       </c>
       <c r="E123" s="5" t="s">
-        <v>1308</v>
+        <v>1310</v>
       </c>
       <c r="F123" s="5" t="s">
         <v>1185</v>
@@ -8535,10 +8600,10 @@
         <v>697</v>
       </c>
       <c r="E127" s="10" t="s">
-        <v>1290</v>
+        <v>1292</v>
       </c>
       <c r="F127" s="10" t="s">
-        <v>1291</v>
+        <v>1293</v>
       </c>
       <c r="G127" s="14"/>
       <c r="H127" s="14"/>
@@ -8561,10 +8626,10 @@
         <v>698</v>
       </c>
       <c r="E128" s="11" t="s">
+        <v>1250</v>
+      </c>
+      <c r="F128" s="11" t="s">
         <v>1248</v>
-      </c>
-      <c r="F128" s="11" t="s">
-        <v>1246</v>
       </c>
       <c r="G128" s="14"/>
       <c r="H128" s="14"/>
@@ -8633,10 +8698,10 @@
         <v>701</v>
       </c>
       <c r="E131" s="5" t="s">
-        <v>1288</v>
+        <v>1290</v>
       </c>
       <c r="F131" s="5" t="s">
-        <v>1266</v>
+        <v>1268</v>
       </c>
       <c r="G131" s="14"/>
       <c r="H131" s="14"/>
@@ -8705,10 +8770,10 @@
         <v>704</v>
       </c>
       <c r="E134" s="12" t="s">
-        <v>1258</v>
+        <v>1260</v>
       </c>
       <c r="F134" s="12" t="s">
-        <v>1259</v>
+        <v>1261</v>
       </c>
       <c r="G134" s="14"/>
       <c r="H134" s="14"/>
@@ -8779,7 +8844,7 @@
         <v>707</v>
       </c>
       <c r="E137" s="5" t="s">
-        <v>1262</v>
+        <v>1264</v>
       </c>
       <c r="F137" s="5" t="s">
         <v>8</v>
@@ -8803,10 +8868,10 @@
         <v>708</v>
       </c>
       <c r="E138" s="12" t="s">
-        <v>1244</v>
+        <v>1246</v>
       </c>
       <c r="F138" s="12" t="s">
-        <v>1234</v>
+        <v>1235</v>
       </c>
       <c r="G138" s="14"/>
       <c r="H138" s="14"/>
@@ -8879,7 +8944,7 @@
         <v>711</v>
       </c>
       <c r="E141" s="5" t="s">
-        <v>1270</v>
+        <v>1272</v>
       </c>
       <c r="F141" s="5" t="s">
         <v>8</v>
@@ -8905,10 +8970,10 @@
         <v>712</v>
       </c>
       <c r="E142" s="5" t="s">
-        <v>1268</v>
+        <v>1270</v>
       </c>
       <c r="F142" s="5" t="s">
-        <v>1269</v>
+        <v>1271</v>
       </c>
       <c r="G142" s="14"/>
       <c r="H142" s="14"/>
@@ -8934,7 +8999,7 @@
         <v>1198</v>
       </c>
       <c r="F143" s="12" t="s">
-        <v>1293</v>
+        <v>1295</v>
       </c>
       <c r="G143" s="14"/>
       <c r="H143" s="14"/>
@@ -8957,7 +9022,7 @@
         <v>714</v>
       </c>
       <c r="E144" s="9" t="s">
-        <v>1235</v>
+        <v>1236</v>
       </c>
       <c r="F144" s="9" t="s">
         <v>8</v>
@@ -8981,7 +9046,7 @@
         <v>715</v>
       </c>
       <c r="E145" s="10" t="s">
-        <v>1264</v>
+        <v>1266</v>
       </c>
       <c r="F145" s="10" t="s">
         <v>1197</v>
@@ -9007,10 +9072,10 @@
         <v>716</v>
       </c>
       <c r="E146" s="12" t="s">
-        <v>1261</v>
+        <v>1263</v>
       </c>
       <c r="F146" s="12" t="s">
-        <v>1260</v>
+        <v>1262</v>
       </c>
       <c r="G146" s="14"/>
       <c r="H146" s="14"/>
@@ -9031,10 +9096,10 @@
         <v>717</v>
       </c>
       <c r="E147" s="12" t="s">
-        <v>1523</v>
+        <v>1234</v>
       </c>
       <c r="F147" s="12" t="s">
-        <v>1234</v>
+        <v>1235</v>
       </c>
       <c r="G147" s="14"/>
       <c r="H147" s="14"/>
@@ -9055,10 +9120,10 @@
         <v>718</v>
       </c>
       <c r="E148" s="5" t="s">
-        <v>1267</v>
+        <v>1269</v>
       </c>
       <c r="F148" s="5" t="s">
-        <v>1266</v>
+        <v>1268</v>
       </c>
       <c r="G148" s="14"/>
       <c r="H148" s="14"/>
@@ -9275,10 +9340,10 @@
         <v>727</v>
       </c>
       <c r="E157" s="9" t="s">
-        <v>1290</v>
+        <v>1292</v>
       </c>
       <c r="F157" s="9" t="s">
-        <v>1291</v>
+        <v>1293</v>
       </c>
       <c r="G157" s="14"/>
       <c r="H157" s="14"/>
@@ -9323,10 +9388,10 @@
         <v>729</v>
       </c>
       <c r="E159" s="7" t="s">
-        <v>1256</v>
+        <v>1258</v>
       </c>
       <c r="F159" s="7" t="s">
-        <v>1255</v>
+        <v>1257</v>
       </c>
       <c r="G159" s="14"/>
       <c r="H159" s="14"/>
@@ -9349,7 +9414,7 @@
         <v>730</v>
       </c>
       <c r="E160" s="10" t="s">
-        <v>1243</v>
+        <v>1245</v>
       </c>
       <c r="F160" s="10" t="s">
         <v>8</v>
@@ -9399,7 +9464,7 @@
         <v>732</v>
       </c>
       <c r="E162" s="9" t="s">
-        <v>1265</v>
+        <v>1267</v>
       </c>
       <c r="F162" s="9" t="s">
         <v>1185</v>
@@ -9473,10 +9538,10 @@
         <v>735</v>
       </c>
       <c r="E165" s="12" t="s">
-        <v>1284</v>
+        <v>1286</v>
       </c>
       <c r="F165" s="12" t="s">
-        <v>1269</v>
+        <v>1271</v>
       </c>
       <c r="G165" s="14" t="s">
         <v>1133</v>
@@ -9681,10 +9746,10 @@
         <v>743</v>
       </c>
       <c r="E173" s="5" t="s">
-        <v>1238</v>
+        <v>1240</v>
       </c>
       <c r="F173" s="5" t="s">
-        <v>1239</v>
+        <v>1241</v>
       </c>
       <c r="G173" s="14"/>
       <c r="H173" s="14"/>
@@ -9757,7 +9822,7 @@
         <v>746</v>
       </c>
       <c r="E176" s="5" t="s">
-        <v>1296</v>
+        <v>1298</v>
       </c>
       <c r="F176" s="5" t="s">
         <v>8</v>
@@ -9781,7 +9846,7 @@
         <v>747</v>
       </c>
       <c r="E177" s="12" t="s">
-        <v>1245</v>
+        <v>1247</v>
       </c>
       <c r="F177" s="12" t="s">
         <v>8</v>
@@ -9804,7 +9869,7 @@
         <v>360</v>
       </c>
       <c r="D178" s="2" t="s">
-        <v>1519</v>
+        <v>1523</v>
       </c>
       <c r="E178" s="9" t="s">
         <v>1176</v>
@@ -9855,10 +9920,10 @@
         <v>749</v>
       </c>
       <c r="E180" s="10" t="s">
-        <v>1288</v>
+        <v>1290</v>
       </c>
       <c r="F180" s="10" t="s">
-        <v>1266</v>
+        <v>1268</v>
       </c>
       <c r="G180" s="14"/>
       <c r="H180" s="14"/>
@@ -9951,7 +10016,7 @@
         <v>753</v>
       </c>
       <c r="E184" s="5" t="s">
-        <v>1252</v>
+        <v>1254</v>
       </c>
       <c r="F184" s="5" t="s">
         <v>8</v>
@@ -10057,10 +10122,10 @@
         <v>757</v>
       </c>
       <c r="E188" s="5" t="s">
-        <v>1254</v>
+        <v>1256</v>
       </c>
       <c r="F188" s="5" t="s">
-        <v>1255</v>
+        <v>1257</v>
       </c>
       <c r="G188" s="14"/>
       <c r="H188" s="14"/>
@@ -10081,7 +10146,7 @@
         <v>758</v>
       </c>
       <c r="E189" s="10" t="s">
-        <v>1271</v>
+        <v>1273</v>
       </c>
       <c r="F189" s="10" t="s">
         <v>8</v>
@@ -10183,7 +10248,7 @@
         <v>762</v>
       </c>
       <c r="E193" s="10" t="s">
-        <v>1272</v>
+        <v>1274</v>
       </c>
       <c r="F193" s="10" t="s">
         <v>8</v>
@@ -10471,7 +10536,7 @@
         <v>773</v>
       </c>
       <c r="E204" s="5" t="s">
-        <v>1295</v>
+        <v>1297</v>
       </c>
       <c r="F204" s="5" t="s">
         <v>8</v>
@@ -10815,10 +10880,10 @@
         <v>786</v>
       </c>
       <c r="E217" s="12" t="s">
-        <v>1274</v>
+        <v>1276</v>
       </c>
       <c r="F217" s="12" t="s">
-        <v>1275</v>
+        <v>1277</v>
       </c>
       <c r="G217" s="14"/>
       <c r="H217" s="14"/>
@@ -10889,7 +10954,7 @@
         <v>789</v>
       </c>
       <c r="E220" s="10" t="s">
-        <v>1289</v>
+        <v>1291</v>
       </c>
       <c r="F220" s="10" t="s">
         <v>8</v>
@@ -10915,10 +10980,10 @@
         <v>790</v>
       </c>
       <c r="E221" s="12" t="s">
-        <v>1247</v>
+        <v>1249</v>
       </c>
       <c r="F221" s="12" t="s">
-        <v>1246</v>
+        <v>1248</v>
       </c>
       <c r="G221" s="14"/>
       <c r="H221" s="14"/>
@@ -10989,7 +11054,7 @@
         <v>793</v>
       </c>
       <c r="E224" s="5" t="s">
-        <v>1265</v>
+        <v>1267</v>
       </c>
       <c r="F224" s="5" t="s">
         <v>1185</v>
@@ -11085,7 +11150,7 @@
         <v>797</v>
       </c>
       <c r="E228" s="5" t="s">
-        <v>1307</v>
+        <v>1309</v>
       </c>
       <c r="F228" s="5" t="s">
         <v>8</v>
@@ -11135,7 +11200,7 @@
         <v>799</v>
       </c>
       <c r="E230" s="12" t="s">
-        <v>1520</v>
+        <v>1239</v>
       </c>
       <c r="F230" s="12" t="s">
         <v>1195</v>
@@ -11182,7 +11247,7 @@
         <v>468</v>
       </c>
       <c r="D232" s="2" t="s">
-        <v>1518</v>
+        <v>1522</v>
       </c>
       <c r="E232" s="7" t="s">
         <v>1179</v>
@@ -11309,10 +11374,10 @@
         <v>805</v>
       </c>
       <c r="E237" s="12" t="s">
-        <v>1299</v>
+        <v>1301</v>
       </c>
       <c r="F237" s="12" t="s">
-        <v>1300</v>
+        <v>1302</v>
       </c>
       <c r="G237" s="14" t="s">
         <v>1133</v>
@@ -11337,7 +11402,7 @@
         <v>806</v>
       </c>
       <c r="E238" s="12" t="s">
-        <v>1283</v>
+        <v>1285</v>
       </c>
       <c r="F238" s="12" t="s">
         <v>8</v>
@@ -11389,10 +11454,10 @@
         <v>808</v>
       </c>
       <c r="E240" s="8" t="s">
+        <v>1259</v>
+      </c>
+      <c r="F240" s="8" t="s">
         <v>1257</v>
-      </c>
-      <c r="F240" s="8" t="s">
-        <v>1255</v>
       </c>
       <c r="G240" s="14"/>
       <c r="H240" s="14" t="s">
@@ -11631,7 +11696,7 @@
         <v>817</v>
       </c>
       <c r="E249" s="10" t="s">
-        <v>1282</v>
+        <v>1284</v>
       </c>
       <c r="F249" s="10" t="s">
         <v>8</v>
@@ -11759,10 +11824,10 @@
         <v>822</v>
       </c>
       <c r="E254" s="10" t="s">
-        <v>1258</v>
+        <v>1260</v>
       </c>
       <c r="F254" s="10" t="s">
-        <v>1259</v>
+        <v>1261</v>
       </c>
       <c r="G254" s="14"/>
       <c r="H254" s="14"/>
@@ -11837,7 +11902,7 @@
         <v>825</v>
       </c>
       <c r="E257" s="10" t="s">
-        <v>1252</v>
+        <v>1254</v>
       </c>
       <c r="F257" s="10" t="s">
         <v>8</v>
@@ -11992,13 +12057,13 @@
         <v>938</v>
       </c>
       <c r="D263" s="2" t="s">
-        <v>1479</v>
+        <v>1483</v>
       </c>
       <c r="E263" s="5" t="s">
-        <v>1480</v>
+        <v>1484</v>
       </c>
       <c r="F263" s="5" t="s">
-        <v>1481</v>
+        <v>1485</v>
       </c>
       <c r="G263" s="14"/>
       <c r="H263" s="14"/>
@@ -12018,10 +12083,10 @@
         <v>940</v>
       </c>
       <c r="D264" s="2" t="s">
-        <v>1430</v>
+        <v>1432</v>
       </c>
       <c r="E264" s="5" t="s">
-        <v>1431</v>
+        <v>1433</v>
       </c>
       <c r="F264" s="5"/>
       <c r="G264" s="14"/>
@@ -12042,10 +12107,10 @@
         <v>942</v>
       </c>
       <c r="D265" s="2" t="s">
-        <v>1357</v>
+        <v>1359</v>
       </c>
       <c r="E265" s="12" t="s">
-        <v>1358</v>
+        <v>1360</v>
       </c>
       <c r="F265" s="12"/>
       <c r="G265" s="14"/>
@@ -12066,13 +12131,13 @@
         <v>944</v>
       </c>
       <c r="D266" s="2" t="s">
+        <v>1445</v>
+      </c>
+      <c r="E266" s="12" t="s">
         <v>1443</v>
       </c>
-      <c r="E266" s="12" t="s">
-        <v>1441</v>
-      </c>
       <c r="F266" s="12" t="s">
-        <v>1442</v>
+        <v>1444</v>
       </c>
       <c r="G266" s="14"/>
       <c r="H266" s="14" t="s">
@@ -12094,10 +12159,10 @@
         <v>946</v>
       </c>
       <c r="D267" s="2" t="s">
-        <v>1514</v>
+        <v>1518</v>
       </c>
       <c r="E267" s="5" t="s">
-        <v>1515</v>
+        <v>1519</v>
       </c>
       <c r="F267" s="5"/>
       <c r="G267" s="14"/>
@@ -12118,10 +12183,10 @@
         <v>948</v>
       </c>
       <c r="D268" s="2" t="s">
-        <v>1353</v>
+        <v>1355</v>
       </c>
       <c r="E268" s="5" t="s">
-        <v>1354</v>
+        <v>1356</v>
       </c>
       <c r="F268" s="5"/>
       <c r="G268" s="14"/>
@@ -12142,10 +12207,10 @@
         <v>950</v>
       </c>
       <c r="D269" s="2" t="s">
-        <v>1510</v>
+        <v>1514</v>
       </c>
       <c r="E269" s="5" t="s">
-        <v>1511</v>
+        <v>1515</v>
       </c>
       <c r="F269" s="5"/>
       <c r="G269" s="14"/>
@@ -12166,10 +12231,10 @@
         <v>952</v>
       </c>
       <c r="D270" s="2" t="s">
-        <v>1496</v>
+        <v>1500</v>
       </c>
       <c r="E270" s="12" t="s">
-        <v>1497</v>
+        <v>1501</v>
       </c>
       <c r="F270" s="12"/>
       <c r="G270" s="14"/>
@@ -12190,13 +12255,13 @@
         <v>954</v>
       </c>
       <c r="D271" s="2" t="s">
+        <v>1371</v>
+      </c>
+      <c r="E271" s="12" t="s">
         <v>1369</v>
       </c>
-      <c r="E271" s="12" t="s">
-        <v>1367</v>
-      </c>
       <c r="F271" s="12" t="s">
-        <v>1366</v>
+        <v>1368</v>
       </c>
       <c r="G271" s="14"/>
       <c r="H271" s="14" t="s">
@@ -12216,10 +12281,10 @@
         <v>956</v>
       </c>
       <c r="D272" s="2" t="s">
-        <v>1416</v>
+        <v>1418</v>
       </c>
       <c r="E272" s="5" t="s">
-        <v>1417</v>
+        <v>1419</v>
       </c>
       <c r="F272" s="5"/>
       <c r="G272" s="14"/>
@@ -12240,13 +12305,13 @@
         <v>958</v>
       </c>
       <c r="D273" s="2" t="s">
-        <v>1436</v>
+        <v>1438</v>
       </c>
       <c r="E273" s="5" t="s">
-        <v>1437</v>
+        <v>1439</v>
       </c>
       <c r="F273" s="5" t="s">
-        <v>1438</v>
+        <v>1440</v>
       </c>
       <c r="G273" s="14"/>
       <c r="H273" s="14"/>
@@ -12266,13 +12331,13 @@
         <v>960</v>
       </c>
       <c r="D274" s="2" t="s">
-        <v>1404</v>
+        <v>1406</v>
       </c>
       <c r="E274" s="12" t="s">
-        <v>1405</v>
+        <v>1407</v>
       </c>
       <c r="F274" s="12" t="s">
-        <v>1406</v>
+        <v>1408</v>
       </c>
       <c r="G274" s="14"/>
       <c r="H274" s="14"/>
@@ -12292,13 +12357,13 @@
         <v>962</v>
       </c>
       <c r="D275" s="2" t="s">
-        <v>1456</v>
+        <v>1459</v>
       </c>
       <c r="E275" s="5" t="s">
-        <v>1522</v>
+        <v>1460</v>
       </c>
       <c r="F275" s="5" t="s">
-        <v>1438</v>
+        <v>1440</v>
       </c>
       <c r="G275" s="14"/>
       <c r="H275" s="14" t="s">
@@ -12318,10 +12383,10 @@
         <v>964</v>
       </c>
       <c r="D276" s="2" t="s">
-        <v>1433</v>
+        <v>1435</v>
       </c>
       <c r="E276" s="5" t="s">
-        <v>1432</v>
+        <v>1434</v>
       </c>
       <c r="F276" s="5"/>
       <c r="G276" s="14"/>
@@ -12340,10 +12405,10 @@
         <v>966</v>
       </c>
       <c r="D277" s="2" t="s">
-        <v>1355</v>
+        <v>1357</v>
       </c>
       <c r="E277" s="5" t="s">
-        <v>1356</v>
+        <v>1358</v>
       </c>
       <c r="F277" s="5"/>
       <c r="G277" s="14"/>
@@ -12362,10 +12427,10 @@
         <v>968</v>
       </c>
       <c r="D278" s="2" t="s">
-        <v>1450</v>
+        <v>1452</v>
       </c>
       <c r="E278" s="5" t="s">
-        <v>1521</v>
+        <v>1453</v>
       </c>
       <c r="F278" s="5"/>
       <c r="G278" s="14"/>
@@ -12386,13 +12451,13 @@
         <v>970</v>
       </c>
       <c r="D279" s="2" t="s">
-        <v>1424</v>
+        <v>1426</v>
       </c>
       <c r="E279" s="10" t="s">
-        <v>1425</v>
+        <v>1427</v>
       </c>
       <c r="F279" s="10" t="s">
-        <v>1426</v>
+        <v>1428</v>
       </c>
       <c r="G279" s="14"/>
       <c r="H279" s="14"/>
@@ -12410,13 +12475,13 @@
         <v>972</v>
       </c>
       <c r="D280" s="2" t="s">
-        <v>1413</v>
+        <v>1415</v>
       </c>
       <c r="E280" s="5" t="s">
-        <v>1415</v>
+        <v>1417</v>
       </c>
       <c r="F280" s="5" t="s">
-        <v>1414</v>
+        <v>1416</v>
       </c>
       <c r="G280" s="14"/>
       <c r="H280" s="14"/>
@@ -12434,10 +12499,10 @@
         <v>974</v>
       </c>
       <c r="D281" s="2" t="s">
-        <v>1319</v>
+        <v>1321</v>
       </c>
       <c r="E281" s="5" t="s">
-        <v>1320</v>
+        <v>1322</v>
       </c>
       <c r="F281" s="5"/>
       <c r="G281" s="14"/>
@@ -12458,10 +12523,10 @@
         <v>976</v>
       </c>
       <c r="D282" s="2" t="s">
-        <v>1512</v>
+        <v>1516</v>
       </c>
       <c r="E282" s="5" t="s">
-        <v>1513</v>
+        <v>1517</v>
       </c>
       <c r="F282" s="5"/>
       <c r="G282" s="14"/>
@@ -12480,10 +12545,10 @@
         <v>978</v>
       </c>
       <c r="D283" s="2" t="s">
-        <v>1411</v>
+        <v>1413</v>
       </c>
       <c r="E283" s="12" t="s">
-        <v>1412</v>
+        <v>1414</v>
       </c>
       <c r="F283" s="12"/>
       <c r="G283" s="14"/>
@@ -12504,10 +12569,10 @@
         <v>980</v>
       </c>
       <c r="D284" s="2" t="s">
-        <v>1315</v>
+        <v>1317</v>
       </c>
       <c r="E284" s="5" t="s">
-        <v>1316</v>
+        <v>1318</v>
       </c>
       <c r="F284" s="5"/>
       <c r="G284" s="14"/>
@@ -12526,10 +12591,10 @@
         <v>982</v>
       </c>
       <c r="D285" s="2" t="s">
-        <v>1325</v>
+        <v>1327</v>
       </c>
       <c r="E285" s="5" t="s">
-        <v>1324</v>
+        <v>1326</v>
       </c>
       <c r="F285" s="5"/>
       <c r="G285" s="14" t="s">
@@ -12552,13 +12617,13 @@
         <v>984</v>
       </c>
       <c r="D286" s="2" t="s">
-        <v>1343</v>
+        <v>1345</v>
       </c>
       <c r="E286" s="12" t="s">
-        <v>1344</v>
+        <v>1346</v>
       </c>
       <c r="F286" s="12" t="s">
-        <v>1345</v>
+        <v>1347</v>
       </c>
       <c r="G286" s="14"/>
       <c r="H286" s="14" t="s">
@@ -12578,10 +12643,10 @@
         <v>986</v>
       </c>
       <c r="D287" s="2" t="s">
-        <v>1409</v>
+        <v>1411</v>
       </c>
       <c r="E287" s="5" t="s">
-        <v>1410</v>
+        <v>1412</v>
       </c>
       <c r="F287" s="5"/>
       <c r="G287" s="14"/>
@@ -12600,10 +12665,10 @@
         <v>988</v>
       </c>
       <c r="D288" s="2" t="s">
-        <v>1500</v>
+        <v>1504</v>
       </c>
       <c r="E288" s="8" t="s">
-        <v>1501</v>
+        <v>1505</v>
       </c>
       <c r="F288" s="8"/>
       <c r="G288" s="14" t="s">
@@ -12624,13 +12689,13 @@
         <v>990</v>
       </c>
       <c r="D289" s="2" t="s">
-        <v>1507</v>
+        <v>1511</v>
       </c>
       <c r="E289" s="5" t="s">
-        <v>1508</v>
+        <v>1512</v>
       </c>
       <c r="F289" s="5" t="s">
-        <v>1509</v>
+        <v>1513</v>
       </c>
       <c r="G289" s="14"/>
       <c r="H289" s="14"/>
@@ -12650,10 +12715,10 @@
         <v>992</v>
       </c>
       <c r="D290" s="2" t="s">
-        <v>1361</v>
+        <v>1363</v>
       </c>
       <c r="E290" s="5" t="s">
-        <v>1360</v>
+        <v>1362</v>
       </c>
       <c r="F290" s="5"/>
       <c r="G290" s="14"/>
@@ -12672,10 +12737,10 @@
         <v>994</v>
       </c>
       <c r="D291" s="2" t="s">
-        <v>1454</v>
+        <v>1457</v>
       </c>
       <c r="E291" s="12" t="s">
-        <v>1455</v>
+        <v>1458</v>
       </c>
       <c r="F291" s="12"/>
       <c r="G291" s="14"/>
@@ -12694,13 +12759,13 @@
         <v>996</v>
       </c>
       <c r="D292" s="2" t="s">
-        <v>1457</v>
+        <v>1461</v>
       </c>
       <c r="E292" s="5" t="s">
-        <v>1458</v>
+        <v>1462</v>
       </c>
       <c r="F292" s="5" t="s">
-        <v>1438</v>
+        <v>1440</v>
       </c>
       <c r="G292" s="14"/>
       <c r="H292" s="14"/>
@@ -12720,10 +12785,10 @@
         <v>998</v>
       </c>
       <c r="D293" s="2" t="s">
-        <v>1439</v>
+        <v>1441</v>
       </c>
       <c r="E293" s="12" t="s">
-        <v>1440</v>
+        <v>1442</v>
       </c>
       <c r="F293" s="12"/>
       <c r="G293" s="14"/>
@@ -12744,10 +12809,10 @@
         <v>1000</v>
       </c>
       <c r="D294" s="2" t="s">
-        <v>1499</v>
+        <v>1503</v>
       </c>
       <c r="E294" s="8" t="s">
-        <v>1498</v>
+        <v>1502</v>
       </c>
       <c r="F294" s="8"/>
       <c r="G294" s="14"/>
@@ -12768,13 +12833,13 @@
         <v>1002</v>
       </c>
       <c r="D295" s="2" t="s">
-        <v>1506</v>
+        <v>1510</v>
       </c>
       <c r="E295" s="5" t="s">
-        <v>1505</v>
+        <v>1509</v>
       </c>
       <c r="F295" s="5" t="s">
-        <v>1504</v>
+        <v>1508</v>
       </c>
       <c r="G295" s="14"/>
       <c r="H295" s="14"/>
@@ -12794,10 +12859,10 @@
         <v>1004</v>
       </c>
       <c r="D296" s="2" t="s">
-        <v>1372</v>
+        <v>1374</v>
       </c>
       <c r="E296" s="12" t="s">
-        <v>1373</v>
+        <v>1375</v>
       </c>
       <c r="F296" s="12"/>
       <c r="G296" s="14"/>
@@ -12818,10 +12883,10 @@
         <v>1006</v>
       </c>
       <c r="D297" s="2" t="s">
-        <v>1378</v>
+        <v>1380</v>
       </c>
       <c r="E297" s="12" t="s">
-        <v>1379</v>
+        <v>1381</v>
       </c>
       <c r="F297" s="12"/>
       <c r="G297" s="14"/>
@@ -12843,7 +12908,7 @@
         <v>1007</v>
       </c>
       <c r="E298" s="5" t="s">
-        <v>1485</v>
+        <v>1489</v>
       </c>
       <c r="F298" s="5"/>
       <c r="G298" s="14"/>
@@ -12862,13 +12927,13 @@
         <v>1010</v>
       </c>
       <c r="D299" s="2" t="s">
-        <v>1476</v>
+        <v>1480</v>
       </c>
       <c r="E299" s="5" t="s">
-        <v>1477</v>
+        <v>1481</v>
       </c>
       <c r="F299" s="5" t="s">
-        <v>1478</v>
+        <v>1482</v>
       </c>
       <c r="G299" s="14"/>
       <c r="H299" s="14" t="s">
@@ -12888,10 +12953,10 @@
         <v>1012</v>
       </c>
       <c r="D300" s="2" t="s">
-        <v>1362</v>
+        <v>1364</v>
       </c>
       <c r="E300" s="5" t="s">
-        <v>1363</v>
+        <v>1365</v>
       </c>
       <c r="F300" s="5"/>
       <c r="G300" s="14"/>
@@ -12912,10 +12977,10 @@
         <v>1014</v>
       </c>
       <c r="D301" s="2" t="s">
-        <v>1335</v>
+        <v>1337</v>
       </c>
       <c r="E301" s="5" t="s">
-        <v>1336</v>
+        <v>1338</v>
       </c>
       <c r="F301" s="5"/>
       <c r="G301" s="14"/>
@@ -12936,10 +13001,10 @@
         <v>1016</v>
       </c>
       <c r="D302" s="2" t="s">
-        <v>1328</v>
+        <v>1330</v>
       </c>
       <c r="E302" s="5" t="s">
-        <v>1329</v>
+        <v>1331</v>
       </c>
       <c r="F302" s="5"/>
       <c r="G302" s="14"/>
@@ -12958,13 +13023,13 @@
         <v>1018</v>
       </c>
       <c r="D303" s="2" t="s">
-        <v>1464</v>
+        <v>1468</v>
       </c>
       <c r="E303" s="5" t="s">
+        <v>1469</v>
+      </c>
+      <c r="F303" s="5" t="s">
         <v>1465</v>
-      </c>
-      <c r="F303" s="5" t="s">
-        <v>1461</v>
       </c>
       <c r="G303" s="14"/>
       <c r="H303" s="14"/>
@@ -12982,10 +13047,10 @@
         <v>1020</v>
       </c>
       <c r="D304" s="2" t="s">
-        <v>1312</v>
+        <v>1314</v>
       </c>
       <c r="E304" s="12" t="s">
-        <v>1311</v>
+        <v>1313</v>
       </c>
       <c r="F304" s="12"/>
       <c r="G304" s="14"/>
@@ -13004,10 +13069,10 @@
         <v>1022</v>
       </c>
       <c r="D305" s="2" t="s">
-        <v>1321</v>
+        <v>1323</v>
       </c>
       <c r="E305" s="5" t="s">
-        <v>1322</v>
+        <v>1324</v>
       </c>
       <c r="F305" s="5"/>
       <c r="G305" s="14"/>
@@ -13028,10 +13093,10 @@
         <v>1024</v>
       </c>
       <c r="D306" s="2" t="s">
-        <v>1444</v>
+        <v>1446</v>
       </c>
       <c r="E306" s="12" t="s">
-        <v>1445</v>
+        <v>1447</v>
       </c>
       <c r="F306" s="12"/>
       <c r="G306" s="14"/>
@@ -13050,13 +13115,13 @@
         <v>1026</v>
       </c>
       <c r="D307" s="2" t="s">
-        <v>1395</v>
+        <v>1397</v>
       </c>
       <c r="E307" s="12" t="s">
-        <v>1396</v>
+        <v>1398</v>
       </c>
       <c r="F307" s="12" t="s">
-        <v>1397</v>
+        <v>1399</v>
       </c>
       <c r="G307" s="14"/>
       <c r="H307" s="14"/>
@@ -13074,13 +13139,13 @@
         <v>1028</v>
       </c>
       <c r="D308" s="2" t="s">
-        <v>1502</v>
+        <v>1506</v>
       </c>
       <c r="E308" s="5" t="s">
-        <v>1503</v>
+        <v>1507</v>
       </c>
       <c r="F308" s="5" t="s">
-        <v>1504</v>
+        <v>1508</v>
       </c>
       <c r="G308" s="14"/>
       <c r="H308" s="14"/>
@@ -13098,10 +13163,10 @@
         <v>1030</v>
       </c>
       <c r="D309" s="2" t="s">
-        <v>1421</v>
+        <v>1423</v>
       </c>
       <c r="E309" s="7" t="s">
-        <v>1420</v>
+        <v>1422</v>
       </c>
       <c r="F309" s="7"/>
       <c r="G309" s="14"/>
@@ -13122,13 +13187,13 @@
         <v>1032</v>
       </c>
       <c r="D310" s="2" t="s">
-        <v>1398</v>
+        <v>1400</v>
       </c>
       <c r="E310" s="12" t="s">
+        <v>1401</v>
+      </c>
+      <c r="F310" s="12" t="s">
         <v>1399</v>
-      </c>
-      <c r="F310" s="12" t="s">
-        <v>1397</v>
       </c>
       <c r="G310" s="14"/>
       <c r="H310" s="14"/>
@@ -13146,13 +13211,13 @@
         <v>1034</v>
       </c>
       <c r="D311" s="2" t="s">
-        <v>1427</v>
+        <v>1429</v>
       </c>
       <c r="E311" s="5" t="s">
-        <v>1428</v>
+        <v>1430</v>
       </c>
       <c r="F311" s="5" t="s">
-        <v>1429</v>
+        <v>1431</v>
       </c>
       <c r="G311" s="14" t="s">
         <v>1133</v>
@@ -13172,10 +13237,10 @@
         <v>1036</v>
       </c>
       <c r="D312" s="2" t="s">
-        <v>1317</v>
+        <v>1319</v>
       </c>
       <c r="E312" s="12" t="s">
-        <v>1318</v>
+        <v>1320</v>
       </c>
       <c r="F312" s="12"/>
       <c r="G312" s="14"/>
@@ -13194,13 +13259,13 @@
         <v>1038</v>
       </c>
       <c r="D313" s="2" t="s">
-        <v>1350</v>
+        <v>1352</v>
       </c>
       <c r="E313" s="5" t="s">
-        <v>1351</v>
+        <v>1353</v>
       </c>
       <c r="F313" s="5" t="s">
-        <v>1352</v>
+        <v>1354</v>
       </c>
       <c r="G313" s="14"/>
       <c r="H313" s="14"/>
@@ -13218,10 +13283,10 @@
         <v>1040</v>
       </c>
       <c r="D314" s="2" t="s">
-        <v>1330</v>
+        <v>1332</v>
       </c>
       <c r="E314" s="5" t="s">
-        <v>1331</v>
+        <v>1333</v>
       </c>
       <c r="F314" s="5"/>
       <c r="G314" s="14"/>
@@ -13240,13 +13305,13 @@
         <v>1042</v>
       </c>
       <c r="D315" s="2" t="s">
-        <v>1370</v>
+        <v>1372</v>
       </c>
       <c r="E315" s="7" t="s">
-        <v>1371</v>
+        <v>1373</v>
       </c>
       <c r="F315" s="7" t="s">
-        <v>1366</v>
+        <v>1368</v>
       </c>
       <c r="G315" s="14" t="s">
         <v>1133</v>
@@ -13266,13 +13331,13 @@
         <v>1044</v>
       </c>
       <c r="D316" s="2" t="s">
-        <v>1332</v>
+        <v>1334</v>
       </c>
       <c r="E316" s="5" t="s">
-        <v>1334</v>
+        <v>1336</v>
       </c>
       <c r="F316" s="5" t="s">
-        <v>1333</v>
+        <v>1335</v>
       </c>
       <c r="G316" s="14"/>
       <c r="H316" s="14" t="s">
@@ -13292,10 +13357,10 @@
         <v>1046</v>
       </c>
       <c r="D317" s="2" t="s">
-        <v>1422</v>
+        <v>1424</v>
       </c>
       <c r="E317" s="5" t="s">
-        <v>1423</v>
+        <v>1425</v>
       </c>
       <c r="F317" s="5"/>
       <c r="G317" s="14"/>
@@ -13314,15 +13379,17 @@
         <v>1048</v>
       </c>
       <c r="D318" s="2" t="s">
-        <v>1472</v>
+        <v>1476</v>
       </c>
       <c r="E318" s="5" t="s">
-        <v>1473</v>
+        <v>1477</v>
       </c>
       <c r="F318" s="5"/>
       <c r="G318" s="14"/>
       <c r="H318" s="14"/>
-      <c r="I318" s="14"/>
+      <c r="I318" s="14" t="s">
+        <v>1133</v>
+      </c>
       <c r="J318" s="14" t="s">
         <v>1133</v>
       </c>
@@ -13338,13 +13405,13 @@
         <v>1050</v>
       </c>
       <c r="D319" s="2" t="s">
-        <v>1400</v>
+        <v>1402</v>
       </c>
       <c r="E319" s="7" t="s">
+        <v>1401</v>
+      </c>
+      <c r="F319" s="7" t="s">
         <v>1399</v>
-      </c>
-      <c r="F319" s="7" t="s">
-        <v>1397</v>
       </c>
       <c r="G319" s="14"/>
       <c r="H319" s="14"/>
@@ -13364,13 +13431,13 @@
         <v>1052</v>
       </c>
       <c r="D320" s="2" t="s">
-        <v>1389</v>
+        <v>1391</v>
       </c>
       <c r="E320" s="5" t="s">
-        <v>1390</v>
+        <v>1392</v>
       </c>
       <c r="F320" s="5" t="s">
-        <v>1391</v>
+        <v>1393</v>
       </c>
       <c r="G320" s="14" t="s">
         <v>1133</v>
@@ -13390,10 +13457,10 @@
         <v>1054</v>
       </c>
       <c r="D321" s="2" t="s">
-        <v>1380</v>
+        <v>1382</v>
       </c>
       <c r="E321" s="12" t="s">
-        <v>1381</v>
+        <v>1383</v>
       </c>
       <c r="F321" s="12"/>
       <c r="G321" s="14"/>
@@ -13412,10 +13479,10 @@
         <v>1056</v>
       </c>
       <c r="D322" s="2" t="s">
-        <v>1337</v>
+        <v>1339</v>
       </c>
       <c r="E322" s="5" t="s">
-        <v>1338</v>
+        <v>1340</v>
       </c>
       <c r="F322" s="5"/>
       <c r="G322" s="14"/>
@@ -13436,10 +13503,10 @@
         <v>1058</v>
       </c>
       <c r="D323" s="2" t="s">
-        <v>1374</v>
+        <v>1376</v>
       </c>
       <c r="E323" s="12" t="s">
-        <v>1375</v>
+        <v>1377</v>
       </c>
       <c r="F323" s="12"/>
       <c r="G323" s="14"/>
@@ -13458,10 +13525,10 @@
         <v>1060</v>
       </c>
       <c r="D324" s="2" t="s">
-        <v>1359</v>
+        <v>1361</v>
       </c>
       <c r="E324" s="5" t="s">
-        <v>1360</v>
+        <v>1362</v>
       </c>
       <c r="F324" s="5"/>
       <c r="G324" s="14" t="s">
@@ -13484,10 +13551,10 @@
         <v>1062</v>
       </c>
       <c r="D325" s="2" t="s">
-        <v>1474</v>
+        <v>1478</v>
       </c>
       <c r="E325" s="12" t="s">
-        <v>1475</v>
+        <v>1479</v>
       </c>
       <c r="F325" s="12"/>
       <c r="G325" s="14"/>
@@ -13506,10 +13573,10 @@
         <v>1064</v>
       </c>
       <c r="D326" s="2" t="s">
-        <v>1376</v>
+        <v>1378</v>
       </c>
       <c r="E326" s="5" t="s">
-        <v>1377</v>
+        <v>1379</v>
       </c>
       <c r="F326" s="5"/>
       <c r="G326" s="14"/>
@@ -13530,13 +13597,13 @@
         <v>1066</v>
       </c>
       <c r="D327" s="2" t="s">
-        <v>1384</v>
+        <v>1386</v>
       </c>
       <c r="E327" s="12" t="s">
-        <v>1385</v>
+        <v>1387</v>
       </c>
       <c r="F327" s="12" t="s">
-        <v>1386</v>
+        <v>1388</v>
       </c>
       <c r="G327" s="14"/>
       <c r="H327" s="14"/>
@@ -13554,10 +13621,10 @@
         <v>1068</v>
       </c>
       <c r="D328" s="2" t="s">
-        <v>1347</v>
+        <v>1349</v>
       </c>
       <c r="E328" s="12" t="s">
-        <v>1346</v>
+        <v>1348</v>
       </c>
       <c r="F328" s="12"/>
       <c r="G328" s="14"/>
@@ -13578,10 +13645,10 @@
         <v>1070</v>
       </c>
       <c r="D329" s="2" t="s">
-        <v>1348</v>
+        <v>1350</v>
       </c>
       <c r="E329" s="12" t="s">
-        <v>1349</v>
+        <v>1351</v>
       </c>
       <c r="F329" s="12"/>
       <c r="G329" s="14" t="s">
@@ -13604,13 +13671,13 @@
         <v>1072</v>
       </c>
       <c r="D330" s="2" t="s">
-        <v>1401</v>
+        <v>1403</v>
       </c>
       <c r="E330" s="5" t="s">
-        <v>1403</v>
+        <v>1405</v>
       </c>
       <c r="F330" s="5" t="s">
-        <v>1402</v>
+        <v>1404</v>
       </c>
       <c r="G330" s="14" t="s">
         <v>1133</v>
@@ -13632,10 +13699,10 @@
         <v>1074</v>
       </c>
       <c r="D331" s="2" t="s">
-        <v>1339</v>
+        <v>1341</v>
       </c>
       <c r="E331" s="12" t="s">
-        <v>1342</v>
+        <v>1344</v>
       </c>
       <c r="F331" s="12"/>
       <c r="G331" s="14" t="s">
@@ -13658,10 +13725,10 @@
         <v>1076</v>
       </c>
       <c r="D332" s="2" t="s">
-        <v>1341</v>
+        <v>1343</v>
       </c>
       <c r="E332" s="12" t="s">
-        <v>1340</v>
+        <v>1342</v>
       </c>
       <c r="F332" s="12"/>
       <c r="G332" s="14"/>
@@ -13682,10 +13749,10 @@
         <v>1078</v>
       </c>
       <c r="D333" s="2" t="s">
-        <v>1491</v>
+        <v>1495</v>
       </c>
       <c r="E333" s="12" t="s">
-        <v>1492</v>
+        <v>1496</v>
       </c>
       <c r="F333" s="12"/>
       <c r="G333" s="14"/>
@@ -13704,17 +13771,15 @@
         <v>1080</v>
       </c>
       <c r="D334" s="2" t="s">
-        <v>1323</v>
+        <v>1325</v>
       </c>
       <c r="E334" s="5" t="s">
-        <v>1324</v>
+        <v>1326</v>
       </c>
       <c r="F334" s="5"/>
       <c r="G334" s="14"/>
       <c r="H334" s="14"/>
-      <c r="I334" s="14" t="s">
-        <v>1133</v>
-      </c>
+      <c r="I334" s="14"/>
       <c r="J334" s="14"/>
     </row>
     <row r="335" spans="1:10" ht="102" customHeight="1">
@@ -13728,13 +13793,13 @@
         <v>1082</v>
       </c>
       <c r="D335" s="2" t="s">
-        <v>1364</v>
+        <v>1366</v>
       </c>
       <c r="E335" s="5" t="s">
-        <v>1365</v>
+        <v>1367</v>
       </c>
       <c r="F335" s="5" t="s">
-        <v>1366</v>
+        <v>1368</v>
       </c>
       <c r="G335" s="14"/>
       <c r="H335" s="14"/>
@@ -13752,10 +13817,10 @@
         <v>1084</v>
       </c>
       <c r="D336" s="2" t="s">
-        <v>1448</v>
+        <v>1450</v>
       </c>
       <c r="E336" s="5" t="s">
-        <v>1449</v>
+        <v>1451</v>
       </c>
       <c r="F336" s="5"/>
       <c r="G336" s="14"/>
@@ -13776,10 +13841,10 @@
         <v>1086</v>
       </c>
       <c r="D337" s="2" t="s">
-        <v>1446</v>
+        <v>1448</v>
       </c>
       <c r="E337" s="5" t="s">
-        <v>1447</v>
+        <v>1449</v>
       </c>
       <c r="F337" s="5"/>
       <c r="G337" s="14"/>
@@ -13800,10 +13865,10 @@
         <v>1088</v>
       </c>
       <c r="D338" s="2" t="s">
-        <v>1326</v>
+        <v>1328</v>
       </c>
       <c r="E338" s="5" t="s">
-        <v>1327</v>
+        <v>1329</v>
       </c>
       <c r="F338" s="5"/>
       <c r="G338" s="14" t="s">
@@ -13826,13 +13891,13 @@
         <v>1090</v>
       </c>
       <c r="D339" s="2" t="s">
-        <v>1469</v>
+        <v>1473</v>
       </c>
       <c r="E339" s="12" t="s">
-        <v>1470</v>
+        <v>1474</v>
       </c>
       <c r="F339" s="12" t="s">
-        <v>1471</v>
+        <v>1475</v>
       </c>
       <c r="G339" s="14"/>
       <c r="H339" s="14"/>
@@ -13850,10 +13915,10 @@
         <v>1092</v>
       </c>
       <c r="D340" s="2" t="s">
-        <v>1313</v>
+        <v>1315</v>
       </c>
       <c r="E340" s="5" t="s">
-        <v>1314</v>
+        <v>1316</v>
       </c>
       <c r="F340" s="5"/>
       <c r="G340" s="14" t="s">
@@ -13876,10 +13941,10 @@
         <v>1094</v>
       </c>
       <c r="D341" s="2" t="s">
-        <v>1516</v>
+        <v>1520</v>
       </c>
       <c r="E341" s="5" t="s">
-        <v>1517</v>
+        <v>1521</v>
       </c>
       <c r="F341" s="5"/>
       <c r="G341" s="14"/>
@@ -13898,13 +13963,13 @@
         <v>1096</v>
       </c>
       <c r="D342" s="2" t="s">
-        <v>1493</v>
+        <v>1497</v>
       </c>
       <c r="E342" s="5" t="s">
-        <v>1494</v>
+        <v>1498</v>
       </c>
       <c r="F342" s="5" t="s">
-        <v>1495</v>
+        <v>1499</v>
       </c>
       <c r="G342" s="14"/>
       <c r="H342" s="14"/>
@@ -13922,10 +13987,10 @@
         <v>1098</v>
       </c>
       <c r="D343" s="2" t="s">
-        <v>1309</v>
+        <v>1311</v>
       </c>
       <c r="E343" s="12" t="s">
-        <v>1310</v>
+        <v>1312</v>
       </c>
       <c r="F343" s="12"/>
       <c r="G343" s="14"/>
@@ -13946,13 +14011,13 @@
         <v>1100</v>
       </c>
       <c r="D344" s="2" t="s">
+        <v>1410</v>
+      </c>
+      <c r="E344" s="8" t="s">
+        <v>1409</v>
+      </c>
+      <c r="F344" s="8" t="s">
         <v>1408</v>
-      </c>
-      <c r="E344" s="8" t="s">
-        <v>1407</v>
-      </c>
-      <c r="F344" s="8" t="s">
-        <v>1406</v>
       </c>
       <c r="G344" s="14"/>
       <c r="H344" s="14"/>
@@ -13970,13 +14035,13 @@
         <v>1102</v>
       </c>
       <c r="D345" s="2" t="s">
-        <v>1392</v>
+        <v>1394</v>
       </c>
       <c r="E345" s="5" t="s">
-        <v>1393</v>
+        <v>1395</v>
       </c>
       <c r="F345" s="5" t="s">
-        <v>1394</v>
+        <v>1396</v>
       </c>
       <c r="G345" s="14"/>
       <c r="H345" s="14"/>
@@ -13994,10 +14059,10 @@
         <v>1104</v>
       </c>
       <c r="D346" s="2" t="s">
-        <v>1383</v>
+        <v>1385</v>
       </c>
       <c r="E346" s="5" t="s">
-        <v>1382</v>
+        <v>1384</v>
       </c>
       <c r="F346" s="5"/>
       <c r="G346" s="14"/>
@@ -14016,10 +14081,10 @@
         <v>1106</v>
       </c>
       <c r="D347" s="2" t="s">
-        <v>1418</v>
+        <v>1420</v>
       </c>
       <c r="E347" s="12" t="s">
-        <v>1419</v>
+        <v>1421</v>
       </c>
       <c r="F347" s="12"/>
       <c r="G347" s="14" t="s">
@@ -14042,13 +14107,13 @@
         <v>1108</v>
       </c>
       <c r="D348" s="2" t="s">
-        <v>1486</v>
+        <v>1490</v>
       </c>
       <c r="E348" s="12" t="s">
-        <v>1487</v>
+        <v>1491</v>
       </c>
       <c r="F348" s="12" t="s">
-        <v>1488</v>
+        <v>1492</v>
       </c>
       <c r="G348" s="14"/>
       <c r="H348" s="14"/>
@@ -14066,13 +14131,13 @@
         <v>1110</v>
       </c>
       <c r="D349" s="2" t="s">
-        <v>1459</v>
+        <v>1463</v>
       </c>
       <c r="E349" s="5" t="s">
-        <v>1460</v>
+        <v>1464</v>
       </c>
       <c r="F349" s="5" t="s">
-        <v>1461</v>
+        <v>1465</v>
       </c>
       <c r="G349" s="14"/>
       <c r="H349" s="14"/>
@@ -14092,13 +14157,13 @@
         <v>1112</v>
       </c>
       <c r="D350" s="2" t="s">
-        <v>1490</v>
+        <v>1494</v>
       </c>
       <c r="E350" s="8" t="s">
-        <v>1489</v>
+        <v>1493</v>
       </c>
       <c r="F350" s="8" t="s">
-        <v>1488</v>
+        <v>1492</v>
       </c>
       <c r="G350" s="14"/>
       <c r="H350" s="14"/>
@@ -14116,13 +14181,13 @@
         <v>1114</v>
       </c>
       <c r="D351" s="2" t="s">
-        <v>1451</v>
+        <v>1454</v>
       </c>
       <c r="E351" s="12" t="s">
-        <v>1452</v>
+        <v>1455</v>
       </c>
       <c r="F351" s="12" t="s">
-        <v>1453</v>
+        <v>1456</v>
       </c>
       <c r="G351" s="14"/>
       <c r="H351" s="14" t="s">
@@ -14142,10 +14207,10 @@
         <v>1116</v>
       </c>
       <c r="D352" s="2" t="s">
-        <v>1434</v>
+        <v>1436</v>
       </c>
       <c r="E352" s="5" t="s">
-        <v>1435</v>
+        <v>1437</v>
       </c>
       <c r="F352" s="5"/>
       <c r="G352" s="14"/>
@@ -14164,13 +14229,13 @@
         <v>1118</v>
       </c>
       <c r="D353" s="2" t="s">
-        <v>1462</v>
+        <v>1466</v>
       </c>
       <c r="E353" s="5" t="s">
-        <v>1463</v>
+        <v>1467</v>
       </c>
       <c r="F353" s="5" t="s">
-        <v>1461</v>
+        <v>1465</v>
       </c>
       <c r="G353" s="14" t="s">
         <v>1133</v>
@@ -14192,10 +14257,10 @@
         <v>1120</v>
       </c>
       <c r="D354" s="2" t="s">
-        <v>1387</v>
+        <v>1389</v>
       </c>
       <c r="E354" s="5" t="s">
-        <v>1388</v>
+        <v>1390</v>
       </c>
       <c r="F354" s="5"/>
       <c r="G354" s="14" t="s">
@@ -14218,13 +14283,13 @@
         <v>1122</v>
       </c>
       <c r="D355" s="2" t="s">
-        <v>1466</v>
+        <v>1470</v>
       </c>
       <c r="E355" s="5" t="s">
-        <v>1467</v>
+        <v>1471</v>
       </c>
       <c r="F355" s="5" t="s">
-        <v>1468</v>
+        <v>1472</v>
       </c>
       <c r="G355" s="14" t="s">
         <v>1133</v>
@@ -14246,13 +14311,13 @@
         <v>1124</v>
       </c>
       <c r="D356" s="2" t="s">
+        <v>1370</v>
+      </c>
+      <c r="E356" s="7" t="s">
+        <v>1369</v>
+      </c>
+      <c r="F356" s="7" t="s">
         <v>1368</v>
-      </c>
-      <c r="E356" s="7" t="s">
-        <v>1367</v>
-      </c>
-      <c r="F356" s="7" t="s">
-        <v>1366</v>
       </c>
       <c r="G356" s="14"/>
       <c r="H356" s="14"/>
@@ -14270,13 +14335,13 @@
         <v>1126</v>
       </c>
       <c r="D357" s="2" t="s">
-        <v>1482</v>
+        <v>1486</v>
       </c>
       <c r="E357" s="5" t="s">
-        <v>1483</v>
+        <v>1487</v>
       </c>
       <c r="F357" s="5" t="s">
-        <v>1484</v>
+        <v>1488</v>
       </c>
       <c r="G357" s="14" t="s">
         <v>1133</v>
@@ -14296,16 +14361,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G39"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="4.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="4.83203125" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="26" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="32" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="44.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="106.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="41.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="7.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="9.109375" style="1"/>
+    <col min="4" max="4" width="44.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="106.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="41.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="132.5" style="1" customWidth="1"/>
+    <col min="8" max="16384" width="9.1640625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="15" customHeight="1">
@@ -15087,70 +15152,114 @@
         <v>8</v>
       </c>
     </row>
-    <row r="35" spans="1:7">
+    <row r="35" spans="1:7" ht="128">
       <c r="A35" s="1">
         <v>1033</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>1127</v>
       </c>
-      <c r="C35" s="2"/>
-      <c r="D35" s="2"/>
+      <c r="C35" s="2" t="s">
+        <v>1535</v>
+      </c>
+      <c r="D35" s="15" t="s">
+        <v>1539</v>
+      </c>
       <c r="E35" s="2"/>
-      <c r="F35" s="2"/>
-      <c r="G35" s="2"/>
-    </row>
-    <row r="36" spans="1:7">
-      <c r="A36" s="1">
+      <c r="F35" s="15" t="s">
+        <v>1541</v>
+      </c>
+      <c r="G35" s="15" t="s">
+        <v>1536</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" ht="128">
+      <c r="A36" s="2">
         <v>1034</v>
       </c>
       <c r="B36" s="2" t="s">
         <v>1128</v>
       </c>
-      <c r="C36" s="2"/>
-      <c r="D36" s="2"/>
+      <c r="C36" s="2" t="s">
+        <v>1534</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>1537</v>
+      </c>
       <c r="E36" s="2"/>
-      <c r="F36" s="2"/>
-      <c r="G36" s="2"/>
-    </row>
-    <row r="37" spans="1:7">
+      <c r="F36" s="15" t="s">
+        <v>1541</v>
+      </c>
+      <c r="G36" s="15" t="s">
+        <v>1536</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" ht="32">
       <c r="A37" s="1">
         <v>1035</v>
       </c>
       <c r="B37" s="2" t="s">
         <v>1129</v>
       </c>
-      <c r="C37" s="2"/>
-      <c r="D37" s="2"/>
-      <c r="E37" s="2"/>
-      <c r="F37" s="2"/>
-      <c r="G37" s="2"/>
-    </row>
-    <row r="38" spans="1:7">
-      <c r="A38" s="1">
+      <c r="C37" s="2" t="s">
+        <v>1525</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>1528</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>1527</v>
+      </c>
+      <c r="F37" s="15" t="s">
+        <v>1529</v>
+      </c>
+      <c r="G37" s="15" t="s">
+        <v>1526</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" ht="64">
+      <c r="A38" s="2">
         <v>1036</v>
       </c>
       <c r="B38" s="2" t="s">
         <v>1130</v>
       </c>
-      <c r="C38" s="2"/>
-      <c r="D38" s="2"/>
-      <c r="E38" s="2"/>
-      <c r="F38" s="2"/>
-      <c r="G38" s="2"/>
-    </row>
-    <row r="39" spans="1:7">
+      <c r="C38" s="2" t="s">
+        <v>1530</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>1531</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>1532</v>
+      </c>
+      <c r="F38" s="15" t="s">
+        <v>1542</v>
+      </c>
+      <c r="G38" s="15" t="s">
+        <v>1540</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" ht="128">
       <c r="A39" s="1">
         <v>1037</v>
       </c>
       <c r="B39" s="2" t="s">
         <v>1131</v>
       </c>
-      <c r="C39" s="2"/>
-      <c r="D39" s="2"/>
+      <c r="C39" s="2" t="s">
+        <v>1533</v>
+      </c>
+      <c r="D39" s="15" t="s">
+        <v>1538</v>
+      </c>
       <c r="E39" s="2"/>
-      <c r="F39" s="2"/>
-      <c r="G39" s="2"/>
+      <c r="F39" s="15" t="s">
+        <v>1541</v>
+      </c>
+      <c r="G39" s="15" t="s">
+        <v>1536</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -15164,11 +15273,11 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="21" style="1" customWidth="1"/>
-    <col min="2" max="2" width="21.44140625" style="1" customWidth="1"/>
-    <col min="3" max="16384" width="9.109375" style="1"/>
+    <col min="2" max="2" width="21.5" style="1" customWidth="1"/>
+    <col min="3" max="16384" width="9.1640625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="15" customHeight="1">
@@ -15211,9 +15320,12 @@
         <v>873</v>
       </c>
     </row>
-    <row r="6" spans="1:2" customFormat="1" ht="14.4">
+    <row r="6" spans="1:2" customFormat="1">
       <c r="A6" t="s">
         <v>1132</v>
+      </c>
+      <c r="B6" t="s">
+        <v>1524</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="15" customHeight="1">

</xml_diff>